<commit_message>
fix: corrige #VALOR! na aba EPI-EPC (referências sem sinal de igual)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018thhqGCNtzAvwRgCiNHzf6
</commit_message>
<xml_diff>
--- a/projetos/fachada-sao-camilo/orcamento/Levantamento_Materiais_Fachada_Sao_Camilo.xlsx
+++ b/projetos/fachada-sao-camilo/orcamento/Levantamento_Materiais_Fachada_Sao_Camilo.xlsx
@@ -8716,10 +8716,9 @@
           <t>par</t>
         </is>
       </c>
-      <c r="D10" s="30" t="inlineStr">
-        <is>
-          <t>Premissas!$C$22</t>
-        </is>
+      <c r="D10" s="30">
+        <f>Premissas!$C$22</f>
+        <v/>
       </c>
       <c r="E10" s="23" t="n">
         <v>145</v>
@@ -8918,10 +8917,9 @@
           <t>un</t>
         </is>
       </c>
-      <c r="D17" s="30" t="inlineStr">
-        <is>
-          <t>Premissas!$C$22</t>
-        </is>
+      <c r="D17" s="30">
+        <f>Premissas!$C$22</f>
+        <v/>
       </c>
       <c r="E17" s="23" t="n">
         <v>38</v>
@@ -9144,10 +9142,9 @@
           <t>pessoa</t>
         </is>
       </c>
-      <c r="D25" s="30" t="inlineStr">
-        <is>
-          <t>Premissas!$C$22</t>
-        </is>
+      <c r="D25" s="30">
+        <f>Premissas!$C$22</f>
+        <v/>
       </c>
       <c r="E25" s="23" t="n">
         <v>260</v>

</xml_diff>